<commit_message>
feat: enhance question handling with input type support and answer processing
</commit_message>
<xml_diff>
--- a/public/question-upload-template.xlsx
+++ b/public/question-upload-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\isolated-two-libs-installer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\isolated-two-libs-installer\WScode\projects\tools_for_admin\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5933AEF9-CCB8-4FAF-9E48-3A540CB4D7E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{625E3EB1-E676-4FB0-A3F1-5A90B90352A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>Код</t>
   </si>
@@ -70,6 +70,24 @@
   </si>
   <si>
     <t>Комментарий к вопросу</t>
+  </si>
+  <si>
+    <t>Какие петли из ассортимента петровича, можно использовать на Стоковых кухнях Вардек</t>
+  </si>
+  <si>
+    <t>multiple_response</t>
+  </si>
+  <si>
+    <t>Samet 90#Clip-on 110#Slide-on 110#Samet 110</t>
+  </si>
+  <si>
+    <t>1#4</t>
+  </si>
+  <si>
+    <t>Random</t>
+  </si>
+  <si>
+    <t>Kitchen_3337</t>
   </si>
 </sst>
 </file>
@@ -126,13 +144,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -414,10 +438,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
     <col min="2" max="2" width="12.28515625" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
     <col min="7" max="7" width="15.140625" customWidth="1"/>
     <col min="8" max="8" width="11.85546875" customWidth="1"/>
     <col min="11" max="11" width="12.28515625" customWidth="1"/>
@@ -475,6 +502,38 @@
       </c>
       <c r="P1" s="1"/>
     </row>
+    <row r="2" spans="1:16" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4">
+        <v>1</v>
+      </c>
+      <c r="K2" s="3"/>
+      <c r="O2" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>